<commit_message>
datos cerrados de yfinance
</commit_message>
<xml_diff>
--- a/config/SP500_yfinance.xlsx
+++ b/config/SP500_yfinance.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Documents\REDALVAROSV14\1 Repositorios para GitHub\3_Portafolio_financiero\src\quant_engine\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Documents\REDALVAROSV14\1 Repositorios para GitHub\3_Portafolio_financiero\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FB2B3C2-1510-4215-B8AA-ABCE8438B8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED182B3-B46C-477A-9012-494E93C7EEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CBB0F558-D610-4D00-9E7B-5B7650BF8105}"/>
+    <workbookView xWindow="210" yWindow="0" windowWidth="21600" windowHeight="11295" xr2:uid="{CBB0F558-D610-4D00-9E7B-5B7650BF8105}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
actualizacion en la base de datos
</commit_message>
<xml_diff>
--- a/config/SP500_yfinance.xlsx
+++ b/config/SP500_yfinance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Documents\REDALVAROSV14\1 Repositorios para GitHub\3_Portafolio financiero\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0BAB080-57F8-43E1-8AF6-827034E5FEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C813970B-9DE0-4668-BD90-BEA2680C3B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="210" yWindow="0" windowWidth="21600" windowHeight="11295" xr2:uid="{CBB0F558-D610-4D00-9E7B-5B7650BF8105}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CBB0F558-D610-4D00-9E7B-5B7650BF8105}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>